<commit_message>
Aggiornata colonna K come richiesto
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111080XXXXXXXX/Lepida/Lepida_CVPI/2.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111080XXXXXXXX/Lepida/Lepida_CVPI/2.1.0/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simone\Desktop\Accreditamento CVPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD670DA3-26F7-4D87-9ED6-A96227AF2ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DBF152-CE48-4D72-95BF-EF10DA7E0197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="206">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -742,9 +742,6 @@
     <t>Trattandosi di un potenziale errore di configurazione del sistema; serve un intervento tecnico manuale per correggere la configurazione e ripristinare il corretto funzionamento del servizio. Non Ã¨ possibile implementare un meccanismo automatico di retry o di invio manuale da parte dell'operatore; in quanto non essendo un errore transitorio; Ã¨ necessario intervenire sulla configurazione del sistema per risolverlo.</t>
   </si>
   <si>
-    <t>Campo valorizzato in modo fisso nel nell'invocazione del servizio</t>
-  </si>
-  <si>
     <t>Si valutano da backoffice le cause del timeout e si procede con intervento risolutivo. Successivamente il client puÃ² procedere con un nuovo tentantivo di invio del documento</t>
   </si>
   <si>
@@ -800,9 +797,6 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.a324eae800^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>Campo valorizzato in modo fisso nel CDA</t>
   </si>
   <si>
     <t>0d2f7fa83f24c4e516b4012bf6460b66</t>
@@ -3030,7 +3024,7 @@
       </c>
       <c r="B2" s="52"/>
       <c r="C2" s="53" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D2" s="52"/>
       <c r="F2" s="6"/>
@@ -3058,7 +3052,7 @@
       </c>
       <c r="B3" s="55"/>
       <c r="C3" s="60" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D3" s="52"/>
       <c r="F3" s="6"/>
@@ -3084,7 +3078,7 @@
       <c r="A4" s="56"/>
       <c r="B4" s="57"/>
       <c r="C4" s="60" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D4" s="52"/>
       <c r="E4" s="4"/>
@@ -3111,7 +3105,7 @@
       <c r="A5" s="58"/>
       <c r="B5" s="59"/>
       <c r="C5" s="60" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D5" s="52"/>
       <c r="F5" s="6"/>
@@ -3357,7 +3351,7 @@
         <v>146</v>
       </c>
       <c r="K11" s="29" t="s">
-        <v>161</v>
+        <v>106</v>
       </c>
       <c r="L11" s="29"/>
       <c r="M11" s="29"/>
@@ -3420,7 +3414,7 @@
         <v>146</v>
       </c>
       <c r="S12" s="29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T12" s="29"/>
       <c r="U12" s="30"/>
@@ -3449,10 +3443,10 @@
         <v>46101</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="H13" s="28" t="s">
         <v>163</v>
-      </c>
-      <c r="H13" s="28" t="s">
-        <v>164</v>
       </c>
       <c r="I13" s="33" t="s">
         <v>157</v>
@@ -3481,7 +3475,7 @@
         <v>58</v>
       </c>
       <c r="S13" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T13" s="29"/>
       <c r="U13" s="30"/>
@@ -3510,13 +3504,13 @@
         <v>46101</v>
       </c>
       <c r="G14" s="28" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H14" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="I14" s="33" t="s">
         <v>166</v>
-      </c>
-      <c r="I14" s="33" t="s">
-        <v>167</v>
       </c>
       <c r="J14" s="29" t="s">
         <v>58</v>
@@ -3542,7 +3536,7 @@
         <v>58</v>
       </c>
       <c r="S14" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T14" s="29"/>
       <c r="U14" s="30"/>
@@ -3571,13 +3565,13 @@
         <v>46101</v>
       </c>
       <c r="G15" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="H15" s="28" t="s">
         <v>168</v>
       </c>
-      <c r="H15" s="28" t="s">
+      <c r="I15" s="33" t="s">
         <v>169</v>
-      </c>
-      <c r="I15" s="33" t="s">
-        <v>170</v>
       </c>
       <c r="J15" s="29" t="s">
         <v>58</v>
@@ -3603,7 +3597,7 @@
         <v>58</v>
       </c>
       <c r="S15" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T15" s="29"/>
       <c r="U15" s="30"/>
@@ -3632,13 +3626,13 @@
         <v>46101</v>
       </c>
       <c r="G16" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H16" s="28" t="s">
+        <v>170</v>
+      </c>
+      <c r="I16" s="33" t="s">
         <v>171</v>
-      </c>
-      <c r="I16" s="33" t="s">
-        <v>172</v>
       </c>
       <c r="J16" s="29" t="s">
         <v>58</v>
@@ -3664,7 +3658,7 @@
         <v>58</v>
       </c>
       <c r="S16" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T16" s="29"/>
       <c r="U16" s="30"/>
@@ -3693,13 +3687,13 @@
         <v>46101</v>
       </c>
       <c r="G17" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="H17" s="28" t="s">
         <v>173</v>
       </c>
-      <c r="H17" s="28" t="s">
+      <c r="I17" s="33" t="s">
         <v>174</v>
-      </c>
-      <c r="I17" s="33" t="s">
-        <v>175</v>
       </c>
       <c r="J17" s="29" t="s">
         <v>58</v>
@@ -3725,7 +3719,7 @@
         <v>58</v>
       </c>
       <c r="S17" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T17" s="29"/>
       <c r="U17" s="30"/>
@@ -3754,13 +3748,13 @@
         <v>46101</v>
       </c>
       <c r="G18" s="28" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H18" s="28" t="s">
+        <v>175</v>
+      </c>
+      <c r="I18" s="33" t="s">
         <v>176</v>
-      </c>
-      <c r="I18" s="33" t="s">
-        <v>177</v>
       </c>
       <c r="J18" s="29" t="s">
         <v>58</v>
@@ -3786,7 +3780,7 @@
         <v>58</v>
       </c>
       <c r="S18" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T18" s="29"/>
       <c r="U18" s="30"/>
@@ -3815,13 +3809,13 @@
         <v>46101</v>
       </c>
       <c r="G19" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="H19" s="28" t="s">
         <v>178</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="I19" s="33" t="s">
         <v>179</v>
-      </c>
-      <c r="I19" s="33" t="s">
-        <v>180</v>
       </c>
       <c r="J19" s="29" t="s">
         <v>58</v>
@@ -3847,7 +3841,7 @@
         <v>58</v>
       </c>
       <c r="S19" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T19" s="29"/>
       <c r="U19" s="30"/>
@@ -3880,7 +3874,7 @@
         <v>146</v>
       </c>
       <c r="K20" s="29" t="s">
-        <v>181</v>
+        <v>106</v>
       </c>
       <c r="L20" s="29"/>
       <c r="M20" s="29"/>
@@ -3919,13 +3913,13 @@
         <v>46101</v>
       </c>
       <c r="G21" s="28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H21" s="28" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="I21" s="33" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="J21" s="29" t="s">
         <v>58</v>
@@ -3951,7 +3945,7 @@
         <v>58</v>
       </c>
       <c r="S21" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T21" s="29"/>
       <c r="U21" s="30"/>
@@ -3980,13 +3974,13 @@
         <v>46101</v>
       </c>
       <c r="G22" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>183</v>
+      </c>
+      <c r="I22" s="33" t="s">
         <v>184</v>
-      </c>
-      <c r="H22" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="I22" s="33" t="s">
-        <v>186</v>
       </c>
       <c r="J22" s="29" t="s">
         <v>58</v>
@@ -4012,7 +4006,7 @@
         <v>58</v>
       </c>
       <c r="S22" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T22" s="29"/>
       <c r="U22" s="30"/>
@@ -4041,13 +4035,13 @@
         <v>46101</v>
       </c>
       <c r="G23" s="28" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H23" s="28" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="I23" s="33" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="J23" s="29" t="s">
         <v>58</v>
@@ -4073,7 +4067,7 @@
         <v>58</v>
       </c>
       <c r="S23" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T23" s="29"/>
       <c r="U23" s="30"/>
@@ -4102,13 +4096,13 @@
         <v>46101</v>
       </c>
       <c r="G24" s="28" t="s">
+        <v>187</v>
+      </c>
+      <c r="H24" s="28" t="s">
+        <v>188</v>
+      </c>
+      <c r="I24" s="33" t="s">
         <v>189</v>
-      </c>
-      <c r="H24" s="28" t="s">
-        <v>190</v>
-      </c>
-      <c r="I24" s="33" t="s">
-        <v>191</v>
       </c>
       <c r="J24" s="29" t="s">
         <v>58</v>
@@ -4134,7 +4128,7 @@
         <v>58</v>
       </c>
       <c r="S24" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T24" s="29"/>
       <c r="U24" s="30"/>
@@ -4163,13 +4157,13 @@
         <v>46101</v>
       </c>
       <c r="G25" s="28" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H25" s="28" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="I25" s="33" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="J25" s="29" t="s">
         <v>58</v>
@@ -4195,7 +4189,7 @@
         <v>58</v>
       </c>
       <c r="S25" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T25" s="29"/>
       <c r="U25" s="30"/>
@@ -4224,13 +4218,13 @@
         <v>46101</v>
       </c>
       <c r="G26" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="H26" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="I26" s="33" t="s">
         <v>194</v>
-      </c>
-      <c r="H26" s="28" t="s">
-        <v>195</v>
-      </c>
-      <c r="I26" s="33" t="s">
-        <v>196</v>
       </c>
       <c r="J26" s="29" t="s">
         <v>58</v>
@@ -4256,7 +4250,7 @@
         <v>58</v>
       </c>
       <c r="S26" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T26" s="29"/>
       <c r="U26" s="30"/>
@@ -4289,7 +4283,7 @@
         <v>146</v>
       </c>
       <c r="K27" s="29" t="s">
-        <v>181</v>
+        <v>106</v>
       </c>
       <c r="L27" s="29"/>
       <c r="M27" s="29"/>
@@ -4332,7 +4326,7 @@
         <v>146</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>181</v>
+        <v>106</v>
       </c>
       <c r="L28" s="27"/>
       <c r="M28" s="29"/>
@@ -4371,13 +4365,13 @@
         <v>46101</v>
       </c>
       <c r="G29" s="28" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H29" s="28" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I29" s="33" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="J29" s="29" t="s">
         <v>58</v>
@@ -4418,13 +4412,13 @@
         <v>46101</v>
       </c>
       <c r="G30" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="H30" s="28" t="s">
+        <v>198</v>
+      </c>
+      <c r="I30" s="33" t="s">
         <v>199</v>
-      </c>
-      <c r="H30" s="28" t="s">
-        <v>200</v>
-      </c>
-      <c r="I30" s="33" t="s">
-        <v>201</v>
       </c>
       <c r="J30" s="29" t="s">
         <v>58</v>
@@ -4465,13 +4459,13 @@
         <v>46101</v>
       </c>
       <c r="G31" s="28" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H31" s="28" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="I31" s="33" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="J31" s="29" t="s">
         <v>58</v>
@@ -9013,12 +9007,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9286,21 +9283,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9325,18 +9328,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Aggiornati file per accreditamento
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111080XXXXXXXX/Lepida/Lepida_CVPI/2.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111080XXXXXXXX/Lepida/Lepida_CVPI/2.1.0/report-checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simone\Desktop\Accreditamento CVPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9935F2D6-EDFC-4B8B-BF7A-E02CEF4D1E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17701A64-04F5-4C6F-98AA-288004F7CE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="600" windowWidth="19440" windowHeight="14880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -751,133 +751,133 @@
     <t>Lepida</t>
   </si>
   <si>
-    <t>2026-04-07T18:40:39Z</t>
-  </si>
-  <si>
-    <t>786ffd10c881f93119910ed6191f3b6b</t>
-  </si>
-  <si>
     <t>Trattandosi di un potenziale errore di configurazione del sistema, serve un intervento tecnico manuale per correggere la configurazione e ripristinare il corretto funzionamento del servizio. Non Ã¨ possibile implementare un meccanismo automatico di retry o di invio manuale da parte dell'operatore, in quanto non essendo un errore transitorio, Ã¨ necessario intervenire sulla configurazione del sistema per risolverlo.</t>
   </si>
   <si>
-    <t>2026-04-07T18:40:40Z</t>
-  </si>
-  <si>
-    <t>ee289fab8dae98ba3ff5f01871749908</t>
-  </si>
-  <si>
-    <t>e7f70f6aa3d4363d260c3c640cf3c88d</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.b31a55bec2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:41Z</t>
-  </si>
-  <si>
-    <t>ba1aca2abb0a6c8c1cf6d4432440a38b</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.3cf04f564e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>d62eed1f28d0c22b593111e1b30f4218</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.279953b1ea^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:42Z</t>
-  </si>
-  <si>
-    <t>ec593b225702d7a59512c0fbf665ce09</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.1b6fa7f13c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>5fa6f6406a3abc7682735d8352b2d538</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.7b162f22b0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:43Z</t>
-  </si>
-  <si>
-    <t>72361002de82a1d64317a4dce9499d3e</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.8d4f01f30e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>9996e6c751d86b6381877afc50e029ca</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.1275ce2518^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:44Z</t>
-  </si>
-  <si>
-    <t>22e25dfe6a76770ed1e75579626e9b99</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.9d8d935530^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>e69048f4fd647be970dcb6631e61c294</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.b0257dd571^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:45Z</t>
-  </si>
-  <si>
-    <t>5a4766c5cb459fdc576191be2f54bf5c</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.82ad7ed288^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:46Z</t>
-  </si>
-  <si>
-    <t>421f6bafa6354df045cb69a7297aa205</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.60a11b925c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>fa0b267ca0d06a72f77d245ee36e3152</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.203ceb09f0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:47Z</t>
-  </si>
-  <si>
-    <t>d0227eb5d117eeed60cf16f8d68d665f</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.0a41b84744^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-04-07T18:40:48Z</t>
-  </si>
-  <si>
-    <t>52dbedf7e13bf57e1592f39428fbf70b</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.b55e65c1ff^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>1cfb772407c14c80471c859ce07a6fe6</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.0ea71b482c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-09T22:38:54Z</t>
+  </si>
+  <si>
+    <t>4c62e776cdc4ec9086c03ccf32de402d</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:38:55Z</t>
+  </si>
+  <si>
+    <t>2ef2431ac9cca36937386d391d1ab25e</t>
+  </si>
+  <si>
+    <t>e75a929fa0f61b00911036ecee8b3e98</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.455dcdbac9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:38:56Z</t>
+  </si>
+  <si>
+    <t>d8521d903675718bf7a6f7abc8842fe2</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.b25c4466a3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>49d9d4633da579238a52321cd3287e65</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.94a5541612^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:38:57Z</t>
+  </si>
+  <si>
+    <t>f564df227aa906f617ced0a8373c9812</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.70729f8974^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>9a577290ce71f73cfd54d8779aa1db20</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.b655c1744e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:38:58Z</t>
+  </si>
+  <si>
+    <t>eb8c1bdbd23fd6526a666be0d6295958</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.9cb2e53a58^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>4f18b9c916c5c76d60a79b2153f942f9</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.bd21df7b8e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:38:59Z</t>
+  </si>
+  <si>
+    <t>6df8759b19cfbb261f68893e428d4ad1</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.3396c4435a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>b65a49ab1da036bba9b5431f206d157b</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.1653218b18^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:39:00Z</t>
+  </si>
+  <si>
+    <t>eaf05afdaaf73d9a6ef854d6f005296d</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.c38fa515fd^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>a41bf917c873952ceb7dc71d89c2d238</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.8b6d0e0dc7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:39:01Z</t>
+  </si>
+  <si>
+    <t>f79a45babc9cd569e752a20b02f60ff7</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.8caee0747e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>c93353317296979c2e017ed3b778e19c</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.73124c0259^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:39:02Z</t>
+  </si>
+  <si>
+    <t>5992211cef2f11da08cbe832276c486b</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.70fd3e2897^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-04-09T22:39:03Z</t>
+  </si>
+  <si>
+    <t>82a8b3f431e5fe5347b0ebe27b58db0e</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.736173ee74d930e556d58b87162a2f32bc02383a123808d438ea8244bfa6a3b9.428362e872^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -3284,13 +3284,13 @@
         <v>45</v>
       </c>
       <c r="F10" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H10" s="28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I10" s="33" t="s">
         <v>155</v>
@@ -3324,7 +3324,7 @@
       <c r="T10" s="29"/>
       <c r="U10" s="30"/>
       <c r="V10" s="31" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="W10" s="29" t="s">
         <v>46</v>
@@ -3443,7 +3443,7 @@
         <v>61</v>
       </c>
       <c r="F13" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G13" s="28" t="s">
         <v>167</v>
@@ -3504,7 +3504,7 @@
         <v>63</v>
       </c>
       <c r="F14" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G14" s="28" t="s">
         <v>167</v>
@@ -3565,7 +3565,7 @@
         <v>65</v>
       </c>
       <c r="F15" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G15" s="28" t="s">
         <v>171</v>
@@ -3626,7 +3626,7 @@
         <v>67</v>
       </c>
       <c r="F16" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G16" s="28" t="s">
         <v>171</v>
@@ -3687,7 +3687,7 @@
         <v>69</v>
       </c>
       <c r="F17" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G17" s="28" t="s">
         <v>176</v>
@@ -3748,7 +3748,7 @@
         <v>71</v>
       </c>
       <c r="F18" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G18" s="28" t="s">
         <v>176</v>
@@ -3809,7 +3809,7 @@
         <v>73</v>
       </c>
       <c r="F19" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G19" s="28" t="s">
         <v>181</v>
@@ -3913,7 +3913,7 @@
         <v>77</v>
       </c>
       <c r="F21" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G21" s="28" t="s">
         <v>181</v>
@@ -3974,7 +3974,7 @@
         <v>79</v>
       </c>
       <c r="F22" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G22" s="28" t="s">
         <v>186</v>
@@ -4035,7 +4035,7 @@
         <v>81</v>
       </c>
       <c r="F23" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G23" s="28" t="s">
         <v>186</v>
@@ -4096,7 +4096,7 @@
         <v>83</v>
       </c>
       <c r="F24" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G24" s="28" t="s">
         <v>191</v>
@@ -4157,16 +4157,16 @@
         <v>85</v>
       </c>
       <c r="F25" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G25" s="28" t="s">
+        <v>191</v>
+      </c>
+      <c r="H25" s="28" t="s">
         <v>194</v>
       </c>
-      <c r="H25" s="28" t="s">
+      <c r="I25" s="33" t="s">
         <v>195</v>
-      </c>
-      <c r="I25" s="33" t="s">
-        <v>196</v>
       </c>
       <c r="J25" s="29" t="s">
         <v>58</v>
@@ -4218,10 +4218,10 @@
         <v>87</v>
       </c>
       <c r="F26" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G26" s="28" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H26" s="28" t="s">
         <v>197</v>
@@ -4365,16 +4365,16 @@
         <v>94</v>
       </c>
       <c r="F29" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G29" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="H29" s="28" t="s">
         <v>199</v>
       </c>
-      <c r="H29" s="28" t="s">
+      <c r="I29" s="33" t="s">
         <v>200</v>
-      </c>
-      <c r="I29" s="33" t="s">
-        <v>201</v>
       </c>
       <c r="J29" s="29" t="s">
         <v>58</v>
@@ -4412,16 +4412,16 @@
         <v>96</v>
       </c>
       <c r="F30" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G30" s="28" t="s">
+        <v>201</v>
+      </c>
+      <c r="H30" s="28" t="s">
         <v>202</v>
       </c>
-      <c r="H30" s="28" t="s">
+      <c r="I30" s="33" t="s">
         <v>203</v>
-      </c>
-      <c r="I30" s="33" t="s">
-        <v>204</v>
       </c>
       <c r="J30" s="29" t="s">
         <v>58</v>
@@ -4459,10 +4459,10 @@
         <v>98</v>
       </c>
       <c r="F31" s="28">
-        <v>46119</v>
+        <v>46121</v>
       </c>
       <c r="G31" s="28" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H31" s="28" t="s">
         <v>205</v>
@@ -9010,6 +9010,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -9273,42 +9294,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD72871-87C6-44C4-AEDE-C35BE2C233EE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9331,9 +9320,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD72871-87C6-44C4-AEDE-C35BE2C233EE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>